<commit_message>
Fix sanitary assignments, stock loan quantities and draft follow-ups
</commit_message>
<xml_diff>
--- a/backend/services/quotation_template.xlsx
+++ b/backend/services/quotation_template.xlsx
@@ -41,11 +41,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="\₹\ #,##0"/>
-    <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0"/>
+    <numFmt numFmtId="164" formatCode="[$₹-en-IN] #,##,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$₹-en-IN] #,##,##0"/>
+    <numFmt numFmtId="166" formatCode="[$₹-en-IN] #,##,##0"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -2056,10 +2056,10 @@
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
@@ -2067,678 +2067,393 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>244475</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>42862</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{305ED83A-AE68-4542-89EA-D2511999E149}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1524000" y="104775"/>
-          <a:ext cx="4816475" cy="1319212"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>381609</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>301595</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2" descr="Grohe Logo PNG Transparent &amp; SVG Vector - Freebie Supply">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13514632-4B44-4567-9FE1-AC7ECDC0E55C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="11025" t="21755" r="12601" b="29719"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="161925" y="1676400"/>
-          <a:ext cx="829284" cy="396845"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>171450</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>542925</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>489925</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>945646</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3" descr="Oyster LifeStyle | Delhi">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D1B6701-22FC-4EB7-A864-59A9FF2B18EF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="14445" t="32127" r="15184" b="31314"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="171450" y="2314575"/>
-          <a:ext cx="928075" cy="402721"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>229209</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>190394</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{291FD7A2-6FE2-440B-818C-77C4C26CF66C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="1447800" y="1704975"/>
-          <a:ext cx="1219809" cy="257069"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>542925</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>121017</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>921869</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5" descr="Qutone Ceramic - The Tiles of India">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E27AD4D-87A3-435A-9D94-19153D594877}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="6662" t="36927" r="2665" b="36485"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="1266825" y="2314575"/>
-          <a:ext cx="1292592" cy="378944"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>581025</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>296619</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>221772</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6" descr="AXOR Brand Launches New Website | 2018-04-03 | phcppros">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E12603D-FE14-4644-8BED-20D5ABF8AFFB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect t="17552" b="20805"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="3019425" y="1638300"/>
-          <a:ext cx="934794" cy="355122"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>495300</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>380756</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>831599</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 7" descr="nexion | Chhabria Tiles">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB899486-39C9-4234-8BEA-8EC826D97275}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
-          <a:biLevel thresh="75000"/>
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="5394" t="27040" r="4531" b="28571"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="2952750" y="2266950"/>
-          <a:ext cx="1085606" cy="336299"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>195828</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>93785</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Picture 8">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A37B914-B6DD-4406-A837-7CE4E0445FCA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4286250" y="1676400"/>
-          <a:ext cx="1395978" cy="189035"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>438150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>106404</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>853777</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Picture 9" descr="Dimore - Apps on Google Play">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A623FF28-E7B4-4D6A-8F8E-EBD0BCF974A4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print">
-          <a:biLevel thresh="75000"/>
-          <a:extLst>
-            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
-              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a14:imgLayer r:embed="rId10">
-                  <a14:imgEffect>
-                    <a14:colorTemperature colorTemp="5900"/>
-                  </a14:imgEffect>
-                </a14:imgLayer>
-              </a14:imgProps>
-            </a:ext>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="1300" t="33665" r="1831" b="33048"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4371975" y="2209800"/>
-          <a:ext cx="1220829" cy="415627"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>289044</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>229906</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Picture 10" descr="Vitra | Brands of the World™ | Download vector logos and logotypes">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC4EFA3E-0EC4-4BFC-B558-D53253E933BB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect t="29931" b="30929"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="6162675" y="1676400"/>
-          <a:ext cx="831969" cy="325156"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>400050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>569120</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>940149</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 11">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6E5A932-0923-4A9D-BCAA-1E4EBBAAA1C1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
-          <a:extLst>
-            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
-              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a14:imgLayer r:embed="rId13">
-                  <a14:imgEffect>
-                    <a14:sharpenSoften amount="25000"/>
-                  </a14:imgEffect>
-                  <a14:imgEffect>
-                    <a14:colorTemperature colorTemp="5900"/>
-                  </a14:imgEffect>
-                  <a14:imgEffect>
-                    <a14:saturation sat="300000"/>
-                  </a14:imgEffect>
-                </a14:imgLayer>
-              </a14:imgProps>
-            </a:ext>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="27643" t="40299" r="24868" b="34525"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="6019800" y="2171700"/>
-          <a:ext cx="1254920" cy="540099"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+<ns0:wsDr xmlns:ns0="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:ns1="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:ns2="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>3</ns0:col>
+      <ns0:colOff>59786</ns0:colOff>
+      <ns0:row>0</ns0:row>
+      <ns0:rowOff>95250</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="4528627" cy="1190625"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="2" name="Picture 1">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{305ED83A-AE68-4542-89EA-D2511999E149}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <ns1:blip ns3:embed="rId1"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr>
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>0</ns0:col>
+      <ns0:colOff>384746</ns0:colOff>
+      <ns0:row>2</ns0:row>
+      <ns0:rowOff>142875</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1040258" cy="428625"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="3" name="Picture 2" descr="Grohe Logo PNG Transparent &amp; SVG Vector - Freebie Supply">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{13514632-4B44-4567-9FE1-AC7ECDC0E55C}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId2"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>0</ns0:col>
+      <ns0:colOff>453859</ns0:colOff>
+      <ns0:row>3</ns0:row>
+      <ns0:rowOff>457200</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="902032" cy="428625"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="4" name="Picture 3" descr="Oyster LifeStyle | Delhi">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{3D1B6701-22FC-4EB7-A864-59A9FF2B18EF}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId3"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>3</ns0:col>
+      <ns0:colOff>4762</ns0:colOff>
+      <ns0:row>3</ns0:row>
+      <ns0:rowOff>21058</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1381125" cy="291258"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="5" name="Picture 4">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{291FD7A2-6FE2-440B-818C-77C4C26CF66C}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <ns1:blip ns3:embed="rId4"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>3</ns0:col>
+      <ns0:colOff>4762</ns0:colOff>
+      <ns0:row>3</ns0:row>
+      <ns0:rowOff>544910</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1381125" cy="253206"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="6" name="Picture 5" descr="Qutone Ceramic - The Tiles of India">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{7E27AD4D-87A3-435A-9D94-19153D594877}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId5"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>5</ns0:col>
+      <ns0:colOff>551189</ns0:colOff>
+      <ns0:row>2</ns0:row>
+      <ns0:rowOff>142875</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1088371" cy="428625"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="7" name="Picture 6" descr="AXOR Brand Launches New Website | 2018-04-03 | phcppros">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{1E12603D-FE14-4644-8BED-20D5ABF8AFFB}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId6"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>5</ns0:col>
+      <ns0:colOff>404812</ns0:colOff>
+      <ns0:row>3</ns0:row>
+      <ns0:rowOff>531848</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1381125" cy="279329"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="8" name="Picture 7" descr="nexion | Chhabria Tiles">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{CB899486-39C9-4234-8BEA-8EC826D97275}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId7"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>8</ns0:col>
+      <ns0:colOff>195262</ns0:colOff>
+      <ns0:row>3</ns0:row>
+      <ns0:rowOff>72031</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1381125" cy="189313"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="9" name="Picture 8">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{7A37B914-B6DD-4406-A837-7CE4E0445FCA}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <ns1:blip ns3:embed="rId8"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>8</ns0:col>
+      <ns0:colOff>195262</ns0:colOff>
+      <ns0:row>3</ns0:row>
+      <ns0:rowOff>513201</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1381125" cy="316622"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="10" name="Picture 9" descr="Dimore - Apps on Google Play">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{A623FF28-E7B4-4D6A-8F8E-EBD0BCF974A4}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId9"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>10</ns0:col>
+      <ns0:colOff>595312</ns0:colOff>
+      <ns0:row>2</ns0:row>
+      <ns0:rowOff>161528</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1381125" cy="391319"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="11" name="Picture 10" descr="Vitra | Brands of the World™ | Download vector logos and logotypes">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{FC4EFA3E-0EC4-4BFC-B558-D53253E933BB}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId11"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+  <ns0:oneCellAnchor>
+    <ns0:from>
+      <ns0:col>11</ns0:col>
+      <ns0:colOff>157715</ns0:colOff>
+      <ns0:row>3</ns0:row>
+      <ns0:rowOff>457200</ns0:rowOff>
+    </ns0:from>
+    <ns0:ext cx="1037119" cy="428625"/>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="12" name="Picture 11">
+          <ns1:extLst>
+            <ns1:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <ns2:creationId id="{B6E5A932-0923-4A9D-BCAA-1E4EBBAAA1C1}"/>
+            </ns1:ext>
+          </ns1:extLst>
+        </ns0:cNvPr>
+        <ns0:cNvPicPr>
+          <ns1:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill rotWithShape="1">
+        <ns1:blip ns3:embed="rId12"/>
+        <ns1:stretch>
+          <ns1:fillRect/>
+        </ns1:stretch>
+      </ns0:blipFill>
+      <ns0:spPr bwMode="auto">
+        <ns1:prstGeom prst="rect">
+          <ns1:avLst/>
+        </ns1:prstGeom>
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:oneCellAnchor>
+</ns0:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>